<commit_message>
Portwell is a pre-AI company
The fixture centred on an AI product, which answered the question the course
asks. Portwell now runs a customer help portal: a self-service site, live since
2019, where customers search the help centre before raising a ticket.

Nothing structural changed. A proposal is a suggestion, deflection is
self-service, and confidence is a match score. The routing rules, the article
eligibility problem and the seeded defects are untouched, because they were
never about the technology.

Both incidents improve. A superseded refund window reaching a customer is now a
knowledge failure rather than a model failure, and correct-in-general advice
reaching the wrong account is a process failure. Those are what a harness fixes.

Word and Excel files were rewritten at zip level, so the reporting pack's stale
cached value survived: it still reports 37.4 per cent attainment where its own
formula computes 36.8.
</commit_message>
<xml_diff>
--- a/docs/data-dictionary.xlsx
+++ b/docs/data-dictionary.xlsx
@@ -565,12 +565,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>staging.proposals</t>
+          <t>staging.suggestions</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>was_deflected</t>
+          <t>was_self-served</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Proposal sent without a human authoring the answer</t>
+          <t>Suggestion sent without a human authoring the answer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -597,7 +597,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>staging.proposals</t>
+          <t>staging.suggestions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -612,12 +612,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Model confidence at proposal time</t>
+          <t>Model confidence at suggestion time</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ops.proposal.confidence</t>
+          <t>ops.suggestion.confidence</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -629,12 +629,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>marts.deflection</t>
+          <t>marts.self_service</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>deflection_rate</t>
+          <t>self_service_rate</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Deflected over closed, per account-month</t>
+          <t>Self-served over closed, per account-month</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>metric deflection_rate v2</t>
+          <t>metric self_service_rate v2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>marts.deflection</t>
+          <t>marts.self_service</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>

<commit_message>
Document the column the rename missed
stock_count_variance was named before the module became Cycle Count in 2024
and was never changed with it. The dictionary now carries it, and says so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data-dictionary.xlsx
+++ b/docs/data-dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="columns" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="columns" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -754,6 +754,38 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>marts.inventory_accuracy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>stock_count_variance</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DECIMAL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Variance found at count, against system quantity</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ops.count_line.variance</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2024-02-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -765,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -789,6 +821,13 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Known gap: the module was renamed to Cycle Count in 2024 and the column name here was not changed with it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>